<commit_message>
Exporta o roteiro em Excel e lista filiais extras de todas as redes.
A aba Excel passa a baixar o roteiro atual, e Locais/planilha passam a
trazer filiais distintas de Ross, Best Buy, Burlington, T.J. Maxx e
outras redes, sem repetir o mesmo endereço em dias diferentes.

Co-authored-by: marcosfcs <marcosfcs@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/public/Roteiro_Orlando_2026.xlsx
+++ b/public/Roteiro_Orlando_2026.xlsx
@@ -601,7 +601,7 @@
         <v>😴 DESCANSO/SONECA — Jantar na I-Drive.</v>
       </c>
       <c r="G6" s="1" t="str">
-        <v>Orlando International Premium Outlets – 4951 International Dr, Orlando, FL 32819 | Orlando Outlet Marketplace – 5269 International Dr | Ross – 5295 International Dr | Five Below – 5295 International Dr, Ste 660 | Ulta – 5295 International Blvd, Ste 100-A (todos em Orlando, FL 32819)</v>
+        <v>Orlando International Premium Outlets – 4951 International Dr, Orlando, FL 32819 | Orlando Outlet Marketplace – 5269 International Dr | Ross – 5295 International Dr | Five Below – 5295 International Dr, Ste 660 | Ulta – 5295 International Blvd, Ste 100-A | T.J. Maxx – 5295 International Dr, Suite 500 (todos em Orlando, FL 32819)</v>
       </c>
       <c r="H6" s="1" t="str">
         <v>International: ~10–15 min | Outlet Marketplace: ~5–10 min</v>
@@ -610,7 +610,7 @@
         <v>Leve o seu carrinho (o outlet também aluga em 5 pontos). Carter's Clearance é apertada para carrinho. Soneca no hotel (10 min).</v>
       </c>
       <c r="J6" s="1" t="str">
-        <v>Horário: seg–sáb 10h–21h, dom 11h–19h. O balcão Simon Guest Services do International fecha ter–qua → pegue os cupons antes, online (Simon / Premium Outlets VIP, grátis). Estacionamento é o ponto fraco: chegar na abertura; valet US$15. Terça depois da Cyber Monday tende a ser mais tranquila que o fim de semana.</v>
+        <v>Horário: seg–sáb 10h–21h, dom 11h–19h. O balcão Simon Guest Services do International fecha ter–qua → pegue os cupons antes, online (Simon / Premium Outlets VIP, grátis). Estacionamento é o ponto fraco: chegar na abertura; valet US$15. Terça depois da Cyber Monday tende a ser mais tranquila que o fim de semana. T.J. Maxx I-Drive fica no mesmo prédio do Ross; outras filiais de Ross/Five Below/Ulta/T.J. Maxx estão na aba Locais.</v>
       </c>
     </row>
     <row r="7">
@@ -732,7 +732,7 @@
         <v>🎡 PASSEIO — Opcional: 'Now Snowing' no Celebration Town Center — neve artificial grátis às 18h (repete 19h, 20h, 21h). Jantar cedo em Celebration e volta.</v>
       </c>
       <c r="G10" s="1" t="str">
-        <v>The Florida Mall (Play Park, Crayola) – 8001 S Orange Blossom Trl, Orlando, FL 32809 | Burlington – 8204 S Orange Blossom Trl | Best Buy – 8350 S Orange Blossom Trl | Celebration Town Center – Market St, Celebration, FL 34747</v>
+        <v>The Florida Mall (Play Park, Crayola) – 8001 S Orange Blossom Trl, Orlando, FL 32809 | Burlington – 8204 S Orange Blossom Trl | Best Buy – 8350 S Orange Blossom Trl | Ross – 1736 Sand Lake Rd, Orlando, FL 32809 | Ulta – 8001 S Orange Blossom Trl, Orlando, FL 32809 | Celebration Town Center – Market St, Celebration, FL 34747</v>
       </c>
       <c r="H10" s="1" t="str">
         <v>Florida Mall: ~10–15 min | Celebration: ~25–30 min</v>
@@ -741,7 +741,7 @@
         <v>Florida Mall tem aluguel de carrinho, banheiros família e fraldário no Dining Pavilion. Ver a neve das 18h e voltar — a festa é amanhã.</v>
       </c>
       <c r="J10" s="1" t="str">
-        <v>Florida Mall no sábado: seg–qui 10h–20h, sex–sáb 10h–21h — chegar na abertura, o shopping lota depois. Gatorland saiu do roteiro (continua na aba "Lugares com criança").</v>
+        <v>Florida Mall no sábado: seg–qui 10h–20h, sex–sáb 10h–21h — chegar na abertura, o shopping lota depois. Gatorland saiu do roteiro (continua na aba "Lugares com criança"). Ross Florida Mall e Ulta Florida Mall ficam no mesmo trecho; Beauty Master Florida Mall é alternativa na aba Locais.</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -834,7 +834,7 @@
         <v>😴 DESCANSO/SONECA — Livre; preparar o dia do Epic Universe.</v>
       </c>
       <c r="G13" s="1" t="str">
-        <v>Target Millenia – 4750 Millenia Plaza Way, Orlando, FL 32839 | Best Buy – 4155 Millenia Blvd | Ross – 4661 Millenia Plaza Way | Marshalls – 4648 Millenia Plaza Way | Ulta – 4600 Millenia Plaza Way Ste 11 | The Mall at Millenia – 4200 Conroy Rd | Nordstrom Rack – 4036 Eastgate Dr, Orlando, FL 32839 (todos em Orlando, FL 32839)</v>
+        <v>Target Millenia – 4750 Millenia Plaza Way, Orlando, FL 32839 | Best Buy – 4155 Millenia Blvd | Ross – 4661 Millenia Plaza Way | Marshalls – 4648 Millenia Plaza Way | Five Below – 4649 Millenia Plaza Way Unit 140 | Ulta – 4600 Millenia Plaza Way Ste 11 | The Mall at Millenia – 4200 Conroy Rd | Nordstrom Rack – 4036 Eastgate Dr, Orlando, FL 32839 (todos em Orlando, FL 32839)</v>
       </c>
       <c r="H13" s="1" t="str">
         <v>~10–15 min (Nordstrom Rack: ~10 min, estimativa)</v>
@@ -843,7 +843,7 @@
         <v>Tudo perto: dá para fazer só a parte da manhã e voltar. Target tem banheiro e lanches para a criança.</v>
       </c>
       <c r="J13" s="1" t="str">
-        <v>Mall at Millenia: seg–sex 11h–21h, sáb 10h–21h, dom 11h–19h (horário de feriado 2026 ainda não publicado). Target e Best Buy: conferir o horário no app. Nordstrom Rack Eastgate: seg–sáb 10h–21h, dom 11h–19h; loja menor que a média, e reviews alertam para devolução rígida (compre o que for ficar).</v>
+        <v>Mall at Millenia: seg–sex 11h–21h, sáb 10h–21h, dom 11h–19h (horário de feriado 2026 ainda não publicado). Target e Best Buy: conferir o horário no app. Nordstrom Rack Eastgate: seg–sáb 10h–21h, dom 11h–19h; loja menor que a média, e reviews alertam para devolução rígida (compre o que for ficar). Five Below Millenia fica no mesmo complexo — não repetir o da I-Drive.</v>
       </c>
     </row>
     <row r="14">
@@ -977,7 +977,7 @@
         <v>Centro de Winter Garden é plano e bom para carrinho. Se a criança dormir no carro na ida, deixe o Beauty Master para a volta, em vez de acordá-la.</v>
       </c>
       <c r="J17" s="1" t="str">
-        <v>Farmers Market: sábado 8h–13h (dado do Google; confirmar no site da cidade, wgfl.gov). Beauty Master é uma loja grande de beleza com seção de K-beauty (não só coreana); reviews são mistos sobre atendimento. Os barcos-cisne do Lake Eola saíram do roteiro. Mercado deste dia: Target Winter Garden Village (e Marshalls no mesmo complexo) — não repetir o Walmart Turkey Lake.</v>
+        <v>Farmers Market: sábado 8h–13h (dado do Google; confirmar no site da cidade, wgfl.gov). Beauty Master é uma loja grande de beleza com seção de K-beauty (não só coreana); reviews são mistos sobre atendimento. Os barcos-cisne do Lake Eola saíram do roteiro. Mercado deste dia: Target Winter Garden Village (e Marshalls no mesmo complexo) — não repetir o Walmart Turkey Lake. Perto do Beauty Master há Ross, Burlington e T.J. Maxx W Colonial; outras filiais de todas as redes estão na aba Locais.</v>
       </c>
     </row>
     <row r="18">
@@ -2286,7 +2286,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J25"/>
+  <dimension ref="A1:J46"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
@@ -3058,39 +3058,711 @@
     </row>
     <row r="25">
       <c r="A25" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B25" s="1" t="str">
+        <v>Ross I-Drive</v>
+      </c>
+      <c r="C25" s="1" t="str">
+        <v>5295 International Dr, Orlando, FL 32819</v>
+      </c>
+      <c r="D25" s="1" t="str">
+        <v>I-Drive</v>
+      </c>
+      <c r="E25" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F25" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G25" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H25" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I25" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J25" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B26" s="1" t="str">
+        <v>Ross Turkey Lake</v>
+      </c>
+      <c r="C26" s="1" t="str">
+        <v>7603 Turkey Lake Rd, Orlando, FL 32819</v>
+      </c>
+      <c r="D26" s="1" t="str">
+        <v>Turkey Lake</v>
+      </c>
+      <c r="E26" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F26" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G26" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H26" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I26" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J26" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B27" s="1" t="str">
+        <v>Ross Millenia</v>
+      </c>
+      <c r="C27" s="1" t="str">
+        <v>4661 Millenia Plaza Way, Orlando, FL 32839</v>
+      </c>
+      <c r="D27" s="1" t="str">
+        <v>Millenia</v>
+      </c>
+      <c r="E27" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F27" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G27" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H27" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I27" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J27" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B28" s="1" t="str">
+        <v>Ross Florida Mall</v>
+      </c>
+      <c r="C28" s="1" t="str">
+        <v>1736 Sand Lake Rd, Orlando, FL 32809</v>
+      </c>
+      <c r="D28" s="1" t="str">
+        <v>Florida Mall</v>
+      </c>
+      <c r="E28" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F28" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G28" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H28" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I28" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J28" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B29" s="1" t="str">
+        <v>Ross Vineland</v>
+      </c>
+      <c r="C29" s="1" t="str">
+        <v>11625 Regency Village Dr, Orlando, FL 32821</v>
+      </c>
+      <c r="D29" s="1" t="str">
+        <v>Vineland</v>
+      </c>
+      <c r="E29" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F29" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G29" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H29" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I29" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J29" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B30" s="1" t="str">
+        <v>Ross W Colonial</v>
+      </c>
+      <c r="C30" s="1" t="str">
+        <v>7445 W Colonial Dr, Orlando, FL 32818</v>
+      </c>
+      <c r="D30" s="1" t="str">
+        <v>W Colonial</v>
+      </c>
+      <c r="E30" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F30" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G30" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H30" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I30" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J30" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B31" s="1" t="str">
+        <v>Best Buy Florida Mall</v>
+      </c>
+      <c r="C31" s="1" t="str">
+        <v>8350 S Orange Blossom Trl, Orlando, FL 32809</v>
+      </c>
+      <c r="D31" s="1" t="str">
+        <v>Florida Mall</v>
+      </c>
+      <c r="E31" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F31" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G31" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H31" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I31" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J31" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B32" s="1" t="str">
+        <v>Best Buy Millenia</v>
+      </c>
+      <c r="C32" s="1" t="str">
+        <v>4155 Millenia Blvd, Orlando, FL 32839</v>
+      </c>
+      <c r="D32" s="1" t="str">
+        <v>Millenia</v>
+      </c>
+      <c r="E32" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F32" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G32" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H32" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I32" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J32" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B33" s="1" t="str">
+        <v>Best Buy Kissimmee</v>
+      </c>
+      <c r="C33" s="1" t="str">
+        <v>1610 W Osceola Pkwy, Kissimmee, FL 34741</v>
+      </c>
+      <c r="D33" s="1" t="str">
+        <v>Kissimmee</v>
+      </c>
+      <c r="E33" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F33" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G33" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H33" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I33" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J33" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B34" s="1" t="str">
+        <v>Burlington Florida Mall</v>
+      </c>
+      <c r="C34" s="1" t="str">
+        <v>8204 S Orange Blossom Trl, Orlando, FL 32809</v>
+      </c>
+      <c r="D34" s="1" t="str">
+        <v>Florida Mall</v>
+      </c>
+      <c r="E34" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F34" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G34" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H34" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I34" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J34" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B35" s="1" t="str">
+        <v>Burlington I-Drive</v>
+      </c>
+      <c r="C35" s="1" t="str">
+        <v>6870 Grand National Dr, Orlando, FL 32819</v>
+      </c>
+      <c r="D35" s="1" t="str">
+        <v>I-Drive</v>
+      </c>
+      <c r="E35" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F35" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G35" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H35" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I35" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J35" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B36" s="1" t="str">
+        <v>Burlington W Colonial</v>
+      </c>
+      <c r="C36" s="1" t="str">
+        <v>7475 W Colonial Dr, Orlando, FL 32818</v>
+      </c>
+      <c r="D36" s="1" t="str">
+        <v>W Colonial</v>
+      </c>
+      <c r="E36" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F36" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G36" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H36" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I36" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J36" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B37" s="1" t="str">
+        <v>Marshalls Millenia</v>
+      </c>
+      <c r="C37" s="1" t="str">
+        <v>4648 Millenia Plaza Way, Orlando, FL 32839</v>
+      </c>
+      <c r="D37" s="1" t="str">
+        <v>Millenia</v>
+      </c>
+      <c r="E37" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F37" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G37" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H37" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I37" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J37" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B38" s="1" t="str">
+        <v>T.J. Maxx I-Drive</v>
+      </c>
+      <c r="C38" s="1" t="str">
+        <v>5295 International Dr, Suite 500, Orlando, FL 32819</v>
+      </c>
+      <c r="D38" s="1" t="str">
+        <v>I-Drive</v>
+      </c>
+      <c r="E38" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F38" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G38" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H38" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I38" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J38" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B39" s="1" t="str">
+        <v>T.J. Maxx Grand National</v>
+      </c>
+      <c r="C39" s="1" t="str">
+        <v>6716 Grand National Dr, Orlando, FL 32819</v>
+      </c>
+      <c r="D39" s="1" t="str">
+        <v>Grand National</v>
+      </c>
+      <c r="E39" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F39" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G39" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H39" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I39" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J39" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B40" s="1" t="str">
+        <v>T.J. Maxx W Colonial</v>
+      </c>
+      <c r="C40" s="1" t="str">
+        <v>7649 W Colonial Dr, Suite 100, Orlando, FL 32818</v>
+      </c>
+      <c r="D40" s="1" t="str">
+        <v>W Colonial</v>
+      </c>
+      <c r="E40" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F40" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G40" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H40" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I40" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J40" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B41" s="1" t="str">
+        <v>T.J. Maxx Rolling Oaks</v>
+      </c>
+      <c r="C41" s="1" t="str">
+        <v>3219 Rolling Oaks Blvd, Kissimmee, FL 34747</v>
+      </c>
+      <c r="D41" s="1" t="str">
+        <v>Rolling Oaks</v>
+      </c>
+      <c r="E41" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F41" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G41" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H41" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I41" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J41" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B42" s="1" t="str">
+        <v>Five Below Millenia</v>
+      </c>
+      <c r="C42" s="1" t="str">
+        <v>4649 Millenia Plaza Way Unit 140, Orlando, FL 32839</v>
+      </c>
+      <c r="D42" s="1" t="str">
+        <v>Millenia</v>
+      </c>
+      <c r="E42" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F42" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G42" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H42" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I42" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J42" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B43" s="1" t="str">
+        <v>Ulta I-Drive</v>
+      </c>
+      <c r="C43" s="1" t="str">
+        <v>5295 International Blvd, Ste 100-A, Orlando, FL 32819</v>
+      </c>
+      <c r="D43" s="1" t="str">
+        <v>I-Drive</v>
+      </c>
+      <c r="E43" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F43" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G43" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H43" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I43" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J43" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B44" s="1" t="str">
+        <v>Ulta Millenia</v>
+      </c>
+      <c r="C44" s="1" t="str">
+        <v>4600 Millenia Plaza Way Ste 11, Orlando, FL 32839</v>
+      </c>
+      <c r="D44" s="1" t="str">
+        <v>Millenia</v>
+      </c>
+      <c r="E44" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F44" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G44" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H44" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I44" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J44" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="str">
+        <v>Compras</v>
+      </c>
+      <c r="B45" s="1" t="str">
+        <v>Ulta Florida Mall</v>
+      </c>
+      <c r="C45" s="1" t="str">
+        <v>8001 S Orange Blossom Trl, Orlando, FL 32809</v>
+      </c>
+      <c r="D45" s="1" t="str">
+        <v>Florida Mall</v>
+      </c>
+      <c r="E45" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="F45" s="1" t="str">
+        <v>a confirmar</v>
+      </c>
+      <c r="G45" s="1" t="str">
+        <v>Filial extra da mesma rede — cada uma tem endereço próprio na aba Locais do app.</v>
+      </c>
+      <c r="H45" s="1" t="str">
+        <v>Não encaixado (alternativa na aba Locais)</v>
+      </c>
+      <c r="I45" s="1" t="str">
+        <v>Aberto</v>
+      </c>
+      <c r="J45" s="1" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="str">
         <v>Já estavam na sua planilha (não repeti): Orlando International e Vineland Premium Outlets, Orlando Outlet Marketplace, Lake Buena Vista Factory Stores, Disney Character Warehouse (Vineland e International), Carter's (inclusive Carter's + OshKosh na LBV Factory Stores).</v>
       </c>
-      <c r="B25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="C25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="D25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="E25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="F25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="G25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="H25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="I25" s="1" t="str">
-        <v/>
-      </c>
-      <c r="J25" s="1" t="str">
+      <c r="B46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="C46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="D46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="E46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="F46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="G46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="H46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="I46" s="1" t="str">
+        <v/>
+      </c>
+      <c r="J46" s="1" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J46"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>